<commit_message>
Petite Cup 47: ZOMAN wins, snaps Maki's 9-cup streak
H2H final: ZOMAN 24.024 over RoundNzt 24.125.
justMaki set the fastest lap of the cup (23.045, R12) but got eliminated
before reaching the final — first non-win since cup 38.

Cup data via parse_petite_log + cup47_screenshot_R1-4.md cross-check.
SGR excluded (tested the map; both mappers otherwise not in lobby).
Map row 3 in xlsx still a placeholder — fill on next edit when map names
are confirmed from cup announcement.

Note: parse_petite_log fell back to COTDTracker-only because
LiveLeaderboardLogger now emits RESULT/LEADERBOARD lines (new schema)
instead of the PROBE_B|SNAPSHOT lines the parser expects. No DNF
overrides needed for this cup (all DNFs in screenshots had no recoverable
times), but the parser should be updated for future cups.
</commit_message>
<xml_diff>
--- a/Petite Cups 46-50.xlsx
+++ b/Petite Cups 46-50.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D44"/>
+  <dimension ref="A2:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -422,6 +422,11 @@
           <t>Petite Cup 46</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Petite Cup 47</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -429,6 +434,11 @@
           <t>Maps: PCDJ #46 - Innominatus by [CSC]OgelGames + PCDJ #46 - Amber Dash by St Nicholas</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Maps: &lt;fill from cup announcement&gt; + &lt;map 2&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -447,6 +457,26 @@
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -464,6 +494,17 @@
       <c r="C6" t="n">
         <v>22.79328</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>24.02438</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -480,6 +521,20 @@
       <c r="D7" t="n">
         <v>17</v>
       </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>24.12512</v>
+      </c>
+      <c r="J7" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -496,6 +551,20 @@
       <c r="D8" t="n">
         <v>16</v>
       </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>23.04567</v>
+      </c>
+      <c r="J8" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -512,6 +581,22 @@
       <c r="D9" t="n">
         <v>15</v>
       </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -528,6 +613,20 @@
       <c r="D10" t="n">
         <v>14</v>
       </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>23.25138</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -544,6 +643,20 @@
       <c r="D11" t="n">
         <v>13</v>
       </c>
+      <c r="G11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>24.25295</v>
+      </c>
+      <c r="J11" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -560,6 +673,20 @@
       <c r="D12" t="n">
         <v>12</v>
       </c>
+      <c r="G12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>23.38956</v>
+      </c>
+      <c r="J12" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -576,6 +703,22 @@
       <c r="D13" t="n">
         <v>12</v>
       </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -592,6 +735,20 @@
       <c r="D14" t="n">
         <v>11</v>
       </c>
+      <c r="G14" t="n">
+        <v>9</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>24.55641</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -608,6 +765,20 @@
       <c r="D15" t="n">
         <v>11</v>
       </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>St Nicholas</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>24.73921</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -624,6 +795,20 @@
       <c r="D16" t="n">
         <v>10</v>
       </c>
+      <c r="G16" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>23.84866</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -640,6 +825,20 @@
       <c r="D17" t="n">
         <v>10</v>
       </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[ZET]Stick</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>24.22853</v>
+      </c>
+      <c r="J17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -656,6 +855,20 @@
       <c r="D18" t="n">
         <v>9</v>
       </c>
+      <c r="G18" t="n">
+        <v>13</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>24.64071</v>
+      </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -672,6 +885,20 @@
       <c r="D19" t="n">
         <v>9</v>
       </c>
+      <c r="G19" t="n">
+        <v>14</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>24.67427</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -688,6 +915,20 @@
       <c r="D20" t="n">
         <v>9</v>
       </c>
+      <c r="G20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>24.82829</v>
+      </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -704,6 +945,22 @@
       <c r="D21" t="n">
         <v>8</v>
       </c>
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -720,6 +977,22 @@
       <c r="D22" t="n">
         <v>8</v>
       </c>
+      <c r="G22" t="n">
+        <v>16</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Jorts</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -736,6 +1009,22 @@
       <c r="D23" t="n">
         <v>8</v>
       </c>
+      <c r="G23" t="n">
+        <v>16</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -752,6 +1041,22 @@
       <c r="D24" t="n">
         <v>7</v>
       </c>
+      <c r="G24" t="n">
+        <v>16</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>[CSC] OccasionallyAmazingGamer</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -768,6 +1073,22 @@
       <c r="D25" t="n">
         <v>7</v>
       </c>
+      <c r="G25" t="n">
+        <v>16</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>[Fenn]Lilly Fenn</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -784,6 +1105,22 @@
       <c r="D26" t="n">
         <v>7</v>
       </c>
+      <c r="G26" t="n">
+        <v>16</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>𝒱V𝑜o𝒾i𝒹d𝒱</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -800,6 +1137,20 @@
       <c r="D27" t="n">
         <v>6</v>
       </c>
+      <c r="G27" t="n">
+        <v>22</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>imagineaclevernamehere</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>25.99005</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -816,6 +1167,22 @@
       <c r="D28" t="n">
         <v>6</v>
       </c>
+      <c r="G28" t="n">
+        <v>23</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -834,6 +1201,22 @@
       <c r="D29" t="n">
         <v>6</v>
       </c>
+      <c r="G29" t="n">
+        <v>23</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -850,6 +1233,22 @@
       <c r="D30" t="n">
         <v>5</v>
       </c>
+      <c r="G30" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[BRED] MrSplatoon07</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -866,6 +1265,22 @@
       <c r="D31" t="n">
         <v>5</v>
       </c>
+      <c r="G31" t="n">
+        <v>25</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -882,6 +1297,22 @@
       <c r="D32" t="n">
         <v>5</v>
       </c>
+      <c r="G32" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>[ZET] zeriv</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -898,6 +1329,22 @@
       <c r="D33" t="n">
         <v>4</v>
       </c>
+      <c r="G33" t="n">
+        <v>25</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>calebmcr</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -914,6 +1361,22 @@
       <c r="D34" t="n">
         <v>4</v>
       </c>
+      <c r="G34" t="n">
+        <v>25</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>mofn</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -932,6 +1395,22 @@
       <c r="D35" t="n">
         <v>4</v>
       </c>
+      <c r="G35" t="n">
+        <v>30</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>[20x]K410K3N</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -948,6 +1427,22 @@
       <c r="D36" t="n">
         <v>3</v>
       </c>
+      <c r="G36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>grop44</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1081,6 +1576,21 @@
         <v>1</v>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>